<commit_message>
docs(report): allinea report alla promozione v4
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -308,7 +308,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>best_a2c_v4 is promotable: it improves big holdout vs heuristic_v1 and beats best_a2c_v3 head-to-head on both big suites. Default/provisioning still need an explicit release decision.</t>
+          <t>best_a2c_v4 is the recommended local/webapp model: it improves big holdout vs heuristic_v1 and beats best_a2c_v3 head-to-head on both big suites. Cloud still needs release asset provisioning.</t>
         </is>
       </c>
     </row>
@@ -432,7 +432,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>promotable</t>
+          <t>promoted</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -445,7 +445,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Promotable candidate; needs explicit release/default decision.</t>
+          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>candidate successor</t>
+          <t>official best</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>promotable</t>
+          <t>promoted</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Promotable candidate; needs explicit release/default decision.</t>
+          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>promotable</t>
+          <t>promoted</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>Create a promotable v4 candidate from the 1M league run.</t>
+          <t>Promote v4 as the recommended local/webapp model.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1357,12 +1357,12 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>promotable</t>
+          <t>promoted</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Create a promotable v4 candidate from the 1M league run.</t>
+          <t>Promote v4 as the recommended local/webapp model.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Ready for maintainer decision on release/default model asset.</t>
+          <t>Frontend/server default now points to v4; cloud still needs release asset provisioning.</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>candidate successor</t>
+          <t>official best</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>promotable</t>
+          <t>promoted</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Promotable candidate; needs explicit release/default decision.</t>
+          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs(piano): aggiorna roadmap e report modelli
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -308,7 +308,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>best_a2c_v4 is the recommended local/webapp model: it improves big holdout vs heuristic_v1 and beats best_a2c_v3 head-to-head on both big suites. Cloud still needs release asset provisioning.</t>
+          <t>best_a2c_v4 is the recommended local/webapp/cloud model: it improves big holdout vs heuristic_v1 and beats best_a2c_v3 head-to-head on both big suites.</t>
         </is>
       </c>
     </row>
@@ -443,9 +443,9 @@
       <c r="D18" s="0">
         <v>1000000</v>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
@@ -969,9 +969,9 @@
           <t>Decision</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t>Promote v4 as the recommended local/webapp model.</t>
+          <t>Promote v4 as the recommended local/webapp/cloud model.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="E7" s="0" t="inlineStr">
         <is>
-          <t>Promote v4 as the recommended local/webapp model.</t>
+          <t>Promote v4 as the recommended local/webapp/cloud model.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Frontend/server default now points to v4; cloud still needs release asset provisioning.</t>
+          <t>Frontend/server/cloud default now points to v4 via release asset provisioning.</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
@@ -1840,9 +1840,9 @@
       <c r="Q5" s="2">
         <v>0.35628</v>
       </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>Promoted as recommended local/webapp model; cloud release asset still required.</t>
+      <c r="R5" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
release(ai): promuovi modello v5
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Detail best_a2c" sheetId="9" r:id="rId9"/>
     <sheet name="Detail best_a2c_v3" sheetId="10" r:id="rId10"/>
     <sheet name="Detail best_a2c_v4" sheetId="11" r:id="rId11"/>
+    <sheet name="Detail best_a2c_v5" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -109,12 +110,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$8</c:f>
+              <c:f>Dashboard!$A$6:$A$9</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$8</c:f>
+              <c:f>Dashboard!$B$6:$B$9</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -196,7 +197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -297,112 +298,103 @@
         <v>0.35628</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>17.832</v>
+      </c>
+      <c r="C9" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.33972</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v4 is the recommended local/webapp/cloud model: it improves big holdout vs heuristic_v1 and beats best_a2c_v3 head-to-head on both big suites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v5 is the recommended v0.11.0 model: it improves big holdout vs heuristic_v1 and beats best_a2c_v4 head-to-head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B14" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C14" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D14" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E14" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D16" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -412,7 +404,7 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D17" s="0">
@@ -420,14 +412,14 @@
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -445,7 +437,57 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
+          <t>Promoted as recommended v3 baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v4</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D19" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
           <t>Promoted as recommended local/webapp/cloud model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D20" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
@@ -1054,9 +1096,309 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>A2C shaped 1.0M game</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v4.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.4}, {"name": "heuristic_v1", "prob": 0.2}, {"name": "heuristic_v2", "prob": 0.3}, {"name": "random", "prob": 0.1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>data/models/bc_v3.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>17.832</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.33972</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>League v5 1M run warm-started from best_a2c_v4 with best_a2c_v4 in the opponent mix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Promote v5 as the recommended model for v0.11.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>It beats best_a2c_v4 head-to-head and improves the heuristic_v1 holdout without material quality regressions.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Big vs best_a2c_v4 +0.34; big vs heuristic_v1 +17.83; decision-quality +18.00, overkill 0.0%, waste 0.07%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1386,14 +1728,59 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Promote v5 as the recommended model for v0.11.0.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>It beats best_a2c_v4 head-to-head and improves the heuristic_v1 holdout without material quality regressions.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Big vs best_a2c_v4 +0.34; big vs heuristic_v1 +17.83; decision-quality +18.00, overkill 0.0%, waste 0.07%.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Frontend/server default now points to v5; cloud rollout needs the v0.11.0 asset URL in env.</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz + a2c_v5_seed401_1m_numba</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I8"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:T6"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1856,14 +2243,100 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>4</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>A2C shaped 1.0M game</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="H6" s="0">
+        <v>310</v>
+      </c>
+      <c r="I6" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="J6" s="0">
+        <v>401</v>
+      </c>
+      <c r="K6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v4.npz</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.4}, {"name": "heuristic_v1", "prob": 0.2}, {"name": "heuristic_v2", "prob": 0.3}, {"name": "random", "prob": 0.1}]</t>
+        </is>
+      </c>
+      <c r="M6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/bc_v3.npz</t>
+        </is>
+      </c>
+      <c r="N6" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="O6" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2">
+        <v>17.832</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0.33972</v>
+      </c>
+      <c r="R6" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>League v5 1M run warm-started from best_a2c_v4 with best_a2c_v4 in the opponent mix.</t>
+        </is>
+      </c>
+      <c r="T6" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T5"/>
+  <autoFilter ref="A1:T6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2802,14 +3275,128 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v5</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G17" s="2">
+        <v>17.832</v>
+      </c>
+      <c r="H17" s="0">
+        <v>72432</v>
+      </c>
+      <c r="I17" s="0">
+        <v>25279</v>
+      </c>
+      <c r="J17" s="0">
+        <v>2289</v>
+      </c>
+      <c r="K17" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+        </is>
+      </c>
+      <c r="M17" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v5</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v4</t>
+        </is>
+      </c>
+      <c r="G18" s="2">
+        <v>0.33972</v>
+      </c>
+      <c r="H18" s="0">
+        <v>49100</v>
+      </c>
+      <c r="I18" s="0">
+        <v>47967</v>
+      </c>
+      <c r="J18" s="0">
+        <v>2933</v>
+      </c>
+      <c r="K18" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
+        </is>
+      </c>
+      <c r="M18" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M16"/>
+  <autoFilter ref="A1:M18"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3007,8 +3594,65 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v5</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G4" s="2">
+        <v>17.99632</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.0006658152686</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/decision_quality_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="M4" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M3"/>
+  <autoFilter ref="A1:M4"/>
 </worksheet>
 </file>
 
@@ -3123,7 +3767,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3459,59 +4103,140 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B14" s="0" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D14" s="0" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E14"/>
+  <autoFilter ref="A1:E17"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
release(ai): promuovi modello v6
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Detail best_a2c_v3" sheetId="10" r:id="rId10"/>
     <sheet name="Detail best_a2c_v4" sheetId="11" r:id="rId11"/>
     <sheet name="Detail best_a2c_v5" sheetId="12" r:id="rId12"/>
+    <sheet name="Detail best_a2c_v6" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -110,12 +111,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$9</c:f>
+              <c:f>Dashboard!$A$6:$A$10</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$9</c:f>
+              <c:f>Dashboard!$B$6:$B$10</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -197,7 +198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -314,112 +315,103 @@
         <v>0.33972</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>18.40148</v>
+      </c>
+      <c r="C10" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.45866</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v5 is the recommended v0.11.0 model: it improves big holdout vs heuristic_v1 and beats best_a2c_v4 head-to-head.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v6 is the recommended v0.12.0 model: the 5M scaling checkpoint improves big holdout vs heuristic_v1 and beats best_a2c_v5 head-to-head on standard and holdout suites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D15" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D17" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -429,7 +421,7 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D18" s="0">
@@ -437,14 +429,14 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -462,14 +454,14 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -487,7 +479,57 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D21" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
           <t>Promoted as recommended model for the v0.11.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D22" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
@@ -1396,9 +1438,309 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6 (league v5 5M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.4}, {"name": "heuristic_v1", "prob": 0.2}, {"name": "heuristic_v2", "prob": 0.3}, {"name": "random", "prob": 0.1}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>data/models/bc_v3.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>18.40148</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.45866</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Scaling v6 5M run warm-started from best_a2c_v5 with best_a2c_v5 in the opponent mix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Promote v6 as the recommended model for v0.12.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>The 1M/3M/5M scaling curve improved monotonically, and the 5M checkpoint beat best_a2c_v5 on both standard and holdout suites without quality regressions.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>5M big vs best_a2c_v5 +0.46; holdout big vs best_a2c_v5 +0.46; big vs heuristic_v1 +18.40; decision-quality +18.58, overkill 0.0%, waste 0.07%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1773,14 +2115,59 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Promote v6 as the recommended model for v0.12.0.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>The 1M/3M/5M scaling curve improved monotonically, and the 5M checkpoint beat best_a2c_v5 on both standard and holdout suites without quality regressions.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>5M big vs best_a2c_v5 +0.46; holdout big vs best_a2c_v5 +0.46; big vs heuristic_v1 +18.40; decision-quality +18.58, overkill 0.0%, waste 0.07%.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Frontend/server default now points to v6; cloud rollout needs the v0.12.0 asset URL in env.</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz + a2c_v6_scaling_seed501_5m_numba</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T7"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2329,14 +2716,100 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>5</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6 (league v5 5M)</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="H7" s="0">
+        <v>310</v>
+      </c>
+      <c r="I7" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="J7" s="0">
+        <v>501</v>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.4}, {"name": "heuristic_v1", "prob": 0.2}, {"name": "heuristic_v2", "prob": 0.3}, {"name": "random", "prob": 0.1}]</t>
+        </is>
+      </c>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t>data/models/bc_v3.npz</t>
+        </is>
+      </c>
+      <c r="N7" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="O7" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" s="2">
+        <v>18.40148</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0.45866</v>
+      </c>
+      <c r="R7" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Scaling v6 5M run warm-started from best_a2c_v5 with best_a2c_v5 in the opponent mix.</t>
+        </is>
+      </c>
+      <c r="T7" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T6"/>
+  <autoFilter ref="A1:T7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M21"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3389,14 +3862,185 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G19" s="2">
+        <v>18.40148</v>
+      </c>
+      <c r="H19" s="0">
+        <v>73177</v>
+      </c>
+      <c r="I19" s="0">
+        <v>24557</v>
+      </c>
+      <c r="J19" s="0">
+        <v>2266</v>
+      </c>
+      <c r="K19" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="M19" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="G20" s="2">
+        <v>0.46138</v>
+      </c>
+      <c r="H20" s="0">
+        <v>49334</v>
+      </c>
+      <c r="I20" s="0">
+        <v>47678</v>
+      </c>
+      <c r="J20" s="0">
+        <v>2988</v>
+      </c>
+      <c r="K20" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_numba.json</t>
+        </is>
+      </c>
+      <c r="M20" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v5_holdout</t>
+        </is>
+      </c>
+      <c r="G21" s="2">
+        <v>0.45866</v>
+      </c>
+      <c r="H21" s="0">
+        <v>49237</v>
+      </c>
+      <c r="I21" s="0">
+        <v>47697</v>
+      </c>
+      <c r="J21" s="0">
+        <v>3066</v>
+      </c>
+      <c r="K21" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
+        </is>
+      </c>
+      <c r="M21" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M18"/>
+  <autoFilter ref="A1:M21"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3651,8 +4295,65 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v6</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G5" s="2">
+        <v>18.58316</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.0007319681727</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="0">
+        <v>100000</v>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/quality_5m_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M4"/>
+  <autoFilter ref="A1:M5"/>
 </worksheet>
 </file>
 
@@ -3767,7 +4468,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4184,59 +4885,140 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B17" s="0" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D17" s="0" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
+  <autoFilter ref="A1:E20"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(ai): usa solver finale come default
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -1440,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1733,14 +1733,41 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>runtime_default</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Make v6 + exact endgame solver the default UI opponent for v0.13.0.</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>The solver is exact, anti-cheat, and effectively free at runtime; it preserves v6 during the game and improves the fully-known endgame instead of trying to distill solver behavior into the network.</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>control_solver(v6) / bc_model_hybrid_endgame equivalence; PIMC max_unknown=0 sweep showed roughly +1.3..+1.6 avg diff vs v6.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E25"/>
+  <autoFilter ref="A1:E26"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2160,8 +2187,53 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>runtime_default</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Make v6 + exact endgame solver the default UI opponent for v0.13.0.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>The solver is exact, anti-cheat, and effectively free at runtime; it preserves v6 during the game and improves the fully-known endgame instead of trying to distill solver behavior into the network.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>control_solver(v6) / bc_model_hybrid_endgame equivalence; PIMC max_unknown=0 sweep showed roughly +1.3..+1.6 avg diff vs v6.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Runtime default changes to bc_model_hybrid_endgame(best_a2c_v6); model progression chart remains unchanged.</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>src/briscola_ai/ai/agents/registry.py + PLAN.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(ai): esponi PIMC come avversario avanzato
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -1440,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1760,14 +1760,41 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>runtime_option</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Expose PIMC(v6, 16x8) as an advanced selectable UI opponent for v0.14.0.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>PIMC adds measurable value over v6 + solver, but costs CPU, so it should be testable by humans without replacing the lower-risk default.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>PIMC(v6,16x10) beat control_solver(v6) at 2000 games; direct Pareto run found no evidence that 16x10 was stronger than 16x8.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:E27"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2232,8 +2259,53 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>runtime_option</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Expose PIMC(v6, 16x8) as an advanced selectable UI opponent for v0.14.0.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>PIMC adds measurable value over v6 + solver, but costs CPU, so it should be testable by humans without replacing the lower-risk default.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>PIMC(v6,16x10) beat control_solver(v6) at 2000 games; direct Pareto run found no evidence that 16x10 was stronger than 16x8.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>UI can select bc_model_pimc_16x8(best_a2c_v6); default remains bc_model_hybrid_endgame(best_a2c_v6).</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>src/briscola_ai/ai/agents/registry.py + scripts/evaluate_pimc.py + PLAN.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I11"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore(release): promuovi best a2c v7
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Detail best_a2c_v4" sheetId="11" r:id="rId11"/>
     <sheet name="Detail best_a2c_v5" sheetId="12" r:id="rId12"/>
     <sheet name="Detail best_a2c_v6" sheetId="13" r:id="rId13"/>
+    <sheet name="Detail best_a2c_v7" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -111,12 +112,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$10</c:f>
+              <c:f>Dashboard!$A$6:$A$11</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$10</c:f>
+              <c:f>Dashboard!$B$6:$B$11</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -198,7 +199,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -331,112 +332,103 @@
         <v>0.45866</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>18.7314</v>
+      </c>
+      <c r="C11" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2.274</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v6 is the recommended v0.12.0 model: the 5M scaling checkpoint improves big holdout vs heuristic_v1 and beats best_a2c_v5 head-to-head on standard and holdout suites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v7 is the recommended v0.19.0 .npz policy: the 5M value-lookahead-opponent A2C run beats best_a2c_v6 head-to-head and improves the v6+solver runtime baseline. The value-lookahead runtime agent remains the stronger advanced option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B16" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C16" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D16" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E16" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D18" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -446,7 +438,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D19" s="0">
@@ -454,14 +446,14 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -479,14 +471,14 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -504,32 +496,82 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D22" s="0">
+        <v>1000000</v>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v6</t>
         </is>
       </c>
-      <c r="B22" s="0" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>promoted</t>
         </is>
       </c>
-      <c r="C22" s="0" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>v3</t>
         </is>
       </c>
-      <c r="D22" s="0">
+      <c r="D23" s="0">
         <v>5000000</v>
       </c>
-      <c r="E22" s="0" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>Promoted as recommended model for the v0.12.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D24" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
         </is>
       </c>
     </row>
@@ -1792,9 +1834,304 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v7 (value-lookahead 5M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260701</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>18.7314</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>2.274</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>5M A2C run warm-started from best_a2c_v6 against the fast Numba value-lookahead opponent. It becomes the default .npz policy; value-lookahead remains the stronger runtime option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>Promote v7 as the recommended .npz policy for v0.19.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>A 5M A2C run against the fast Numba value-lookahead opponent produced a policy that beats v6 head-to-head and also improves the v6+solver runtime baseline.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout vs best_a2c_v6 +2.27; medium candidate+solver vs v6+solver +2.27; big holdout vs heuristic_v1 +18.73. It remains slightly below v6 value-lookahead runtime (-0.64 on 10k), so value-lookahead stays selectable as the advanced option.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2304,14 +2641,59 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>Promote v7 as the recommended .npz policy for v0.19.0.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>A 5M A2C run against the fast Numba value-lookahead opponent produced a policy that beats v6 head-to-head and also improves the v6+solver runtime baseline.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout vs best_a2c_v6 +2.27; medium candidate+solver vs v6+solver +2.27; big holdout vs heuristic_v1 +18.73. It remains slightly below v6 value-lookahead runtime (-0.64 on 10k), so value-lookahead stays selectable as the advanced option.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Frontend/server/cloud default model moves to best_a2c_v7; value model asset remains unchanged.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz + train_a2c fast_numba_determinized value-lookahead screen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:I12"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:T8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2946,8 +3328,89 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>6</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v7 (value-lookahead 5M)</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="H8" s="0">
+        <v>310</v>
+      </c>
+      <c r="I8" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="J8" s="0">
+        <v>20260701</v>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
+        </is>
+      </c>
+      <c r="L8" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N8" s="2">
+        <v>0</v>
+      </c>
+      <c r="O8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" s="2">
+        <v>18.7314</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>2.274</v>
+      </c>
+      <c r="R8" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>5M A2C run warm-started from best_a2c_v6 against the fast Numba value-lookahead opponent. It becomes the default .npz policy; value-lookahead remains the stronger runtime option.</t>
+        </is>
+      </c>
+      <c r="T8" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T7"/>
+  <autoFilter ref="A1:T8"/>
 </worksheet>
 </file>
 
@@ -4612,7 +5075,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -5110,59 +5573,140 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>data/eval_best_a2c_v7_vs_heuristic_v1_big_holdout_seedrange1000000.json</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>data/eval_a2c_vs_value_lookahead_5M_vs_v6_big_holdout_seedrange1000000.json</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B20" s="0" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D20" s="0" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:E23"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore(release): promuovi best a2c v8
best_a2c_v8.npz = encoder v4 (memoria delle prese) + Net2Net hidden 256,
catena: v7 -> pad v4 -> 5M A2C vs value-lookahead(v7) -> widening
128->256 -> altre 5M. Gate (big holdout 100k, CI su coppie):
vs best_a2c_v7 +0.89 (CI +0.74..+1.05); vs heuristic_v1 +17.61.

- default UI/server/cloud -> best_a2c_v8.npz (primo default v4 e 256);
- value model invariato; value-lookahead resta opzione avanzata (nota:
  nelle simulazioni determinizzate il blocco memoria v4 della base e'
  vuoto, degradazione lieve);
- report modelli rigenerato: Dashboard con curva fino a v8 (range
  grafico verificato);
- versione 0.22.0.
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Detail best_a2c_v5" sheetId="12" r:id="rId12"/>
     <sheet name="Detail best_a2c_v6" sheetId="13" r:id="rId13"/>
     <sheet name="Detail best_a2c_v7" sheetId="14" r:id="rId14"/>
+    <sheet name="Detail best_a2c_v8" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -112,12 +113,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$11</c:f>
+              <c:f>Dashboard!$A$6:$A$12</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$11</c:f>
+              <c:f>Dashboard!$B$6:$B$12</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -199,7 +200,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -348,112 +349,103 @@
         <v>2.274</v>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>17.6067</v>
+      </c>
+      <c r="C12" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.893</v>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v7 is the recommended v0.19.0 .npz policy: the 5M value-lookahead-opponent A2C run beats best_a2c_v6 head-to-head and improves the v6+solver runtime baseline. The value-lookahead runtime agent remains the stronger advanced option.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v8 is the recommended v0.22.0 .npz policy: encoder v4 (trick-history memory) plus Net2Net widening to hidden 256, trained via two ExIt sparring generations against value-lookahead(v7). It beats best_a2c_v7 head-to-head (+0.89, 100k paired). The value-lookahead runtime agent remains the stronger advanced option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B17" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C17" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D17" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E17" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D19" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -463,7 +455,7 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D20" s="0">
@@ -471,14 +463,14 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -496,14 +488,14 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -521,14 +513,14 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -542,18 +534,18 @@
         </is>
       </c>
       <c r="D23" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -571,7 +563,57 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D25" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
           <t>Promoted as recommended model for the v0.19.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D26" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
         </is>
       </c>
     </row>
@@ -2129,9 +2171,304 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v8 (v4 + net2net 256, 10M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260715</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/exit_iter2_seed_v4_h256.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>17.6067</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.893</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Encoder v4 (trick-history features) + Net2Net widening to hidden 256. Chain: warm-start from best_a2c_v7 (v4 zero-pad), 5M A2C games vs value-lookahead(v7), widening 128-&gt;256, 5M more games. Beats best_a2c_v7 head-to-head (+0.89, CI +0.74..+1.05, 100k paired); the lower score vs heuristic_v1 relative to v7 (17.61 vs 18.73) reflects style non-transitivity, not regression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Promote v8 (encoder v4 + hidden 256) as the recommended .npz policy for v0.22.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>The ExIt iteration-1/2 arms measured every student-side lever with paired controls: the v4 trick-history features add +0.27 net (first positive runtime evidence of the encoder program), Net2Net capacity adds a marginal +0.18, and the combined chain beats v7 by +0.89.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout 100k paired CIs: vs best_a2c_v7 +0.89 (CI +0.74..+1.05); vs iter1-v4 +0.18 (CI +0.03..+0.33); vs heuristic_v1 +17.61. Belief-as-policy-input was killed (-0.56 vs its own init): the belief is a deterministic function of the same v4 features, so as policy input it is redundant and gradient-chasing it erodes tuned instinct.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2686,14 +3023,59 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Promote v8 (encoder v4 + hidden 256) as the recommended .npz policy for v0.22.0.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>The ExIt iteration-1/2 arms measured every student-side lever with paired controls: the v4 trick-history features add +0.27 net (first positive runtime evidence of the encoder program), Net2Net capacity adds a marginal +0.18, and the combined chain beats v7 by +0.89.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout 100k paired CIs: vs best_a2c_v7 +0.89 (CI +0.74..+1.05); vs iter1-v4 +0.18 (CI +0.03..+0.33); vs heuristic_v1 +17.61. Belief-as-policy-input was killed (-0.56 vs its own init): the belief is a deterministic function of the same v4 features, so as policy input it is redundant and gradient-chasing it erodes tuned instinct.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Frontend/server/cloud default model moves to best_a2c_v8 (first v4-encoder, first hidden-256 default); value model asset unchanged. Known nuance: inside value-lookahead determinized simulations the v4 history block is empty (mild degradation of the advanced opponent's response modeling, not a correctness issue).</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz + ExIt iteration-1/2 (docs/plans/belief-expert-iteration.md)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
+  <autoFilter ref="A1:I13"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T9"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3409,8 +3791,89 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v8 (v4 + net2net 256, 10M)</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H9" s="0">
+        <v>369</v>
+      </c>
+      <c r="I9" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="J9" s="0">
+        <v>20260715</v>
+      </c>
+      <c r="K9" s="0" t="inlineStr">
+        <is>
+          <t>data/models/exit_iter2_seed_v4_h256.npz</t>
+        </is>
+      </c>
+      <c r="L9" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" s="2">
+        <v>0</v>
+      </c>
+      <c r="O9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2">
+        <v>17.6067</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0.893</v>
+      </c>
+      <c r="R9" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>Encoder v4 (trick-history features) + Net2Net widening to hidden 256. Chain: warm-start from best_a2c_v7 (v4 zero-pad), 5M A2C games vs value-lookahead(v7), widening 128-&gt;256, 5M more games. Beats best_a2c_v7 head-to-head (+0.89, CI +0.74..+1.05, 100k paired); the lower score vs heuristic_v1 relative to v7 (17.61 vs 18.73) reflects style non-transitivity, not regression.</t>
+        </is>
+      </c>
+      <c r="T9" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T8"/>
+  <autoFilter ref="A1:T9"/>
 </worksheet>
 </file>
 
@@ -5075,7 +5538,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -5654,59 +6117,140 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_heuristic_v1_big.json</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_v7_big.json</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B23" s="0" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D23" s="0" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E23"/>
+  <autoFilter ref="A1:E26"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix(report): indice di forza cumulato nel grafico di progressione
Il grafico plottava solo il punteggio vs heuristic_v1 (metro fisso ma
DEBOLE): per non-transitivita' di stile v8 vi appare sotto v7 pur
battendolo head-to-head (+0.89). Aggiunta la colonna e la seconda
serie 'Cumulative strength index' (somma dei margini h2h generazione
su generazione): monotona per costruzione quando ogni promozione
batte il predecessore, e' il metro onesto della progressione.
Report rigenerato.
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -122,6 +122,27 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Cumulative strength index (sum of H2H)</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="7"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$6:$A$12</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$E$6:$E$12</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
         <c:axId val="100"/>
         <c:axId val="101"/>
       </c:lineChart>
@@ -252,6 +273,11 @@
           <t>H2H big holdout vs predecessor/current best</t>
         </is>
       </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Cumulative strength index (sum of H2H)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -268,6 +294,9 @@
       <c r="D6" s="2">
         <v>0.76442</v>
       </c>
+      <c r="E6" s="2">
+        <v>0.764</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -284,6 +313,9 @@
       <c r="D7" s="2">
         <v>0.17928</v>
       </c>
+      <c r="E7" s="2">
+        <v>0.944</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -300,6 +332,9 @@
       <c r="D8" s="2">
         <v>0.35628</v>
       </c>
+      <c r="E8" s="2">
+        <v>1.3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -316,6 +351,9 @@
       <c r="D9" s="2">
         <v>0.33972</v>
       </c>
+      <c r="E9" s="2">
+        <v>1.64</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -332,6 +370,9 @@
       <c r="D10" s="2">
         <v>0.45866</v>
       </c>
+      <c r="E10" s="2">
+        <v>2.098</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -348,6 +389,9 @@
       <c r="D11" s="2">
         <v>2.274</v>
       </c>
+      <c r="E11" s="2">
+        <v>4.372</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -363,6 +407,9 @@
       </c>
       <c r="D12" s="2">
         <v>0.893</v>
+      </c>
+      <c r="E12" s="2">
+        <v>5.265</v>
       </c>
     </row>
     <row r="13"/>

</xml_diff>

<commit_message>
fix(report): legenda del grafico leggibile
Nomi delle serie compatti ('vs heuristic_v1 (metro fisso)' e 'Indice
cumulato (somma H2H)'), font esplicito 11pt, overlay disattivato e
riquadro del grafico allargato (16 colonne x 26 righe): la legenda in
basso non risulta piu' schiacciata/troncata. Report rigenerato.
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -105,7 +105,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Big holdout vs heuristic_v1</c:v>
+            <c:v>vs heuristic_v1 (metro fisso)</c:v>
           </c:tx>
           <c:marker>
             <c:symbol val="circle"/>
@@ -126,7 +126,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Cumulative strength index (sum of H2H)</c:v>
+            <c:v>Indice cumulato (somma H2H)</c:v>
           </c:tx>
           <c:marker>
             <c:symbol val="diamond"/>
@@ -178,6 +178,17 @@
     <c:legend>
       <c:legendPos val="b"/>
       <c:layout/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1100"/>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
@@ -194,9 +205,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">

</xml_diff>

<commit_message>
chore(release): promuovi best a2c v9 — versione 0.26.0
best_a2c_v9.npz = 'super training' 20M partite vs cartellone misto
(value-lookahead(v8) 65%, v8 specchio 15%, euristiche+random 20% —
ricetta del mix proposta dal maintainer). Gate (big 100k, CI coppie):
- vs best_a2c_v8: +0.97 (CI +0.82..+1.12);
- vs heuristic_v1: +18.78 — RECORD assoluto: prima promozione che
  migliora entrambi i metri (non-transitivita' di stile sanata);
- testa a testa col braccio di controllo (maestro PIMC d'elite, 5M):
  +0.63 (CI +0.48..+0.78) — volume+varieta' battono il maestro.

- default UI/server/cloud -> best_a2c_v9.npz;
- report modelli rigenerato (curva a 8 modelli, entrambe le serie in
  crescita; range grafico verificato);
- diario di bordo: nuovo capitolo 11 'I due allievi' + approfondimento
  docs/diario/11-due-allievi.md + genealogia aggiornata;
- README/PLAN allineati. Versione 0.26.0.
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -21,6 +21,7 @@
     <sheet name="Detail best_a2c_v6" sheetId="13" r:id="rId13"/>
     <sheet name="Detail best_a2c_v7" sheetId="14" r:id="rId14"/>
     <sheet name="Detail best_a2c_v8" sheetId="15" r:id="rId15"/>
+    <sheet name="Detail best_a2c_v9" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -113,12 +114,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$12</c:f>
+              <c:f>Dashboard!$A$6:$A$13</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$12</c:f>
+              <c:f>Dashboard!$B$6:$B$13</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -134,12 +135,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$12</c:f>
+              <c:f>Dashboard!$A$6:$A$13</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$E$6:$E$12</c:f>
+              <c:f>Dashboard!$E$6:$E$13</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -232,7 +233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -423,112 +424,106 @@
         <v>5.265</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="0" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="C13" s="0">
+        <v>20000000</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.97</v>
+      </c>
+      <c r="E13" s="2">
+        <v>6.235</v>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v8 is the recommended v0.22.0 .npz policy: encoder v4 (trick-history memory) plus Net2Net widening to hidden 256, trained via two ExIt sparring generations against value-lookahead(v7). It beats best_a2c_v7 head-to-head (+0.89, 100k paired). The value-lookahead runtime agent remains the stronger advanced option.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v9 is the recommended v0.26.0 .npz policy: a 20M-game super training vs a mixed panel (value-lookahead(v8), mirror, heuristics). It beats v8 head-to-head (+0.97) and sets the heuristic_v1 record (+18.78) - the first model improving on both meters. The value-lookahead runtime agent remains the stronger advanced option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B18" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C18" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D18" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E18" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D20" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -538,7 +533,7 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D21" s="0">
@@ -546,14 +541,14 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -571,14 +566,14 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -596,14 +591,14 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -617,18 +612,18 @@
         </is>
       </c>
       <c r="D24" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -646,14 +641,14 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.19.0 release.</t>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
+          <t>best_a2c_v7</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -663,7 +658,7 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D26" s="0">
@@ -671,7 +666,57 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D27" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
           <t>Promoted as recommended model for the v0.22.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D28" s="0">
+        <v>20000000</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
         </is>
       </c>
     </row>
@@ -2524,9 +2569,304 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v9 (20M mix, v4+256)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260720</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.65}, {"name": "heuristic_v1", "prob": 0.06}, {"name": "heuristic_v2", "prob": 0.1}, {"name": "random", "prob": 0.04}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>18.78</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>20M-game 'super training' vs a mixed panel: value-lookahead(v8) 65%, v8 mirror 15%, heuristics+random 20% (the 'bar' share, maintainer's recipe). Beats v8 +0.97 head-to-head AND sets the heuristic_v1 record (+18.78): first model that improves on BOTH meters. Also beats the PIMC-teacher arm (5M vs the strongest master) by +0.63: volume+variety won over elite teaching in this regime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Promote v9 (20M mixed-panel super training) as the recommended .npz policy for v0.26.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Two-arm experiment: 20M games vs mixed panel (VL(v8) 65%, mirror 15%, heuristics+random 20%) vs 5M games vs the strongest teacher (PIMC belief 32x10). Volume+variety won on every axis.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Arm A vs v8: +0.97 (CI +0.82..+1.12, 100k paired); vs heuristic_v1: +18.78 (all-time record); head-to-head vs arm B: +0.63 (CI +0.48..+0.78). Arm B (elite teacher) reached only +0.40 vs v8 and regressed vs heuristic_v1 (16.71): monotone diet erodes anti-weak style.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3126,14 +3466,59 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Promote v9 (20M mixed-panel super training) as the recommended .npz policy for v0.26.0.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Two-arm experiment: 20M games vs mixed panel (VL(v8) 65%, mirror 15%, heuristics+random 20%) vs 5M games vs the strongest teacher (PIMC belief 32x10). Volume+variety won on every axis.</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Arm A vs v8: +0.97 (CI +0.82..+1.12, 100k paired); vs heuristic_v1: +18.78 (all-time record); head-to-head vs arm B: +0.63 (CI +0.48..+0.78). Arm B (elite teacher) reached only +0.40 vs v8 and regressed vs heuristic_v1 (16.71): monotone diet erodes anti-weak style.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Default model moves to best_a2c_v9; first promotion that improves BOTH progression meters simultaneously (no style non-transitivity to explain). Mix recipe credited to the maintainer.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz + two-arm super training (data/exit/due_bracci.log)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:I14"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T10"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3930,8 +4315,89 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>8</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v9 (20M mix, v4+256)</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H10" s="0">
+        <v>369</v>
+      </c>
+      <c r="I10" s="0">
+        <v>20000000</v>
+      </c>
+      <c r="J10" s="0">
+        <v>20260720</v>
+      </c>
+      <c r="K10" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.65}, {"name": "heuristic_v1", "prob": 0.06}, {"name": "heuristic_v2", "prob": 0.1}, {"name": "random", "prob": 0.04}]</t>
+        </is>
+      </c>
+      <c r="N10" s="2">
+        <v>0</v>
+      </c>
+      <c r="O10" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2">
+        <v>18.78</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0.97</v>
+      </c>
+      <c r="R10" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>20M-game 'super training' vs a mixed panel: value-lookahead(v8) 65%, v8 mirror 15%, heuristics+random 20% (the 'bar' share, maintainer's recipe). Beats v8 +0.97 head-to-head AND sets the heuristic_v1 record (+18.78): first model that improves on BOTH meters. Also beats the PIMC-teacher arm (5M vs the strongest master) by +0.63: volume+variety won over elite teaching in this regime.</t>
+        </is>
+      </c>
+      <c r="T10" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T9"/>
+  <autoFilter ref="A1:T10"/>
 </worksheet>
 </file>
 
@@ -5596,7 +6062,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6256,59 +6722,140 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/superA_vs_h1_big.json</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v9</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/superA_vs_v8_big.json</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B26" s="0" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D26" s="0" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E26"/>
+  <autoFilter ref="A1:E29"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore(release): promuovi best a2c v10 — versione 0.27.0
best_a2c_v10.npz = il 'giocatore definitivo': 30M partite contro il
cartellone completo (maestro PIMC belief 25%, value-lookahead 35%,
specchio 15%, euristiche+random 25% — dosi del maintainer, base v9).

Gate (big 100k, CI coppie):
- vs best_a2c_v9: +0.66 (CI +0.51..+0.81);
- vs heuristic_v1: +20.52 — RECORD assoluto (era 18.78): entrambi i
  metri della progressione al massimo storico.

Nota onesta registrata ovunque: rendimenti decrescenti confermati
(+0.97 -> +0.66 per generazione): l'asintoto del gioco a due e' vicino.

- default UI/server/cloud -> best_a2c_v10.npz;
- report rigenerato (9 modelli, entrambe le curve al massimo);
- diario: capitolo 12 'Il cartellone completo' + approfondimento
  12-giocatore-definitivo.md + serie campioni aggiornata;
- README/PLAN allineati. Versione 0.27.0.
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Detail best_a2c_v7" sheetId="14" r:id="rId14"/>
     <sheet name="Detail best_a2c_v8" sheetId="15" r:id="rId15"/>
     <sheet name="Detail best_a2c_v9" sheetId="16" r:id="rId16"/>
+    <sheet name="Detail best_a2c_v10" sheetId="17" r:id="rId17"/>
   </sheets>
 </workbook>
 </file>
@@ -114,12 +115,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$13</c:f>
+              <c:f>Dashboard!$A$6:$A$14</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$13</c:f>
+              <c:f>Dashboard!$B$6:$B$14</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -135,12 +136,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$13</c:f>
+              <c:f>Dashboard!$A$6:$A$14</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$E$6:$E$13</c:f>
+              <c:f>Dashboard!$E$6:$E$14</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -233,7 +234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -443,112 +444,106 @@
         <v>6.235</v>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>20.52</v>
+      </c>
+      <c r="C14" s="0">
+        <v>30000000</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.66</v>
+      </c>
+      <c r="E14" s="2">
+        <v>6.895</v>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v9 is the recommended v0.26.0 .npz policy: a 20M-game super training vs a mixed panel (value-lookahead(v8), mirror, heuristics). It beats v8 head-to-head (+0.97) and sets the heuristic_v1 record (+18.78) - the first model improving on both meters. The value-lookahead runtime agent remains the stronger advanced option.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v10 is the recommended v0.27.0 .npz policy: a 30M-game run vs the complete panel (PIMC-belief teacher, value-lookahead, mirror, heuristics). It beats v9 (+0.66) and sets the all-time heuristic_v1 record (+20.52): both meters at their maximum. The value-lookahead runtime agent remains the stronger advanced option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B19" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C19" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D19" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D21" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -558,7 +553,7 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D22" s="0">
@@ -566,14 +561,14 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -591,14 +586,14 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -616,14 +611,14 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -637,18 +632,18 @@
         </is>
       </c>
       <c r="D25" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -666,14 +661,14 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.19.0 release.</t>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
+          <t>best_a2c_v7</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -683,7 +678,7 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D27" s="0">
@@ -691,32 +686,82 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.22.0 release.</t>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
+          <t>best_a2c_v8</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D28" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v9</t>
         </is>
       </c>
-      <c r="B28" s="0" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>promoted</t>
         </is>
       </c>
-      <c r="C28" s="0" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>v4</t>
         </is>
       </c>
-      <c r="D28" s="0">
+      <c r="D29" s="0">
         <v>20000000</v>
       </c>
-      <c r="E28" s="0" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>Promoted as recommended model for the v0.26.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D30" s="0">
+        <v>30000000</v>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
         </is>
       </c>
     </row>
@@ -2864,9 +2909,304 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v10.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v10 (30M cartellone completo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>30000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260722</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_pimc_belief", "prob": 0.25}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.35}, {"name": "heuristic_v1", "prob": 0.08}, {"name": "heuristic_v2", "prob": 0.12}, {"name": "random", "prob": 0.05}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>20.52</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>The 'definitive' 30M-game run vs the complete panel: PIMC-belief teacher 25%, value-lookahead 35%, mirror 15%, heuristics+random 25%, all on v9 base (panel doses by the maintainer). Beats v9 +0.66 head-to-head and sets a new all-time heuristic_v1 record (+20.52, up from 18.78): both progression meters at their maximum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Promote v10 (30M complete-panel run) as the recommended .npz policy for v0.27.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Combines every lesson from the two-arm experiment: volume, variety, the elite PIMC-belief teacher at the per-game-efficient dose (25%), and a 25% heuristics share to keep anti-weak style.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout 100k paired CIs: vs best_a2c_v9 +0.66 (CI +0.51..+0.81); vs heuristic_v1 +20.52 (record, previous 18.78). Diminishing returns visible (+0.97 -&gt; +0.66 per generation despite more games and a better teacher): the asymptote is near.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3511,14 +3851,59 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Promote v10 (30M complete-panel run) as the recommended .npz policy for v0.27.0.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Combines every lesson from the two-arm experiment: volume, variety, the elite PIMC-belief teacher at the per-game-efficient dose (25%), and a 25% heuristics share to keep anti-weak style.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Big holdout 100k paired CIs: vs best_a2c_v9 +0.66 (CI +0.51..+0.81); vs heuristic_v1 +20.52 (record, previous 18.78). Diminishing returns visible (+0.97 -&gt; +0.66 per generation despite more games and a better teacher): the asymptote is near.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Default model moves to best_a2c_v10; both progression meters at all-time highs.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v10.npz + 30M complete-panel run (data/exit/definitivo.log)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:I15"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:T11"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4396,8 +4781,89 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v10.npz</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v10 (30M cartellone completo)</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H11" s="0">
+        <v>369</v>
+      </c>
+      <c r="I11" s="0">
+        <v>30000000</v>
+      </c>
+      <c r="J11" s="0">
+        <v>20260722</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v9.npz</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_pimc_belief", "prob": 0.25}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.35}, {"name": "heuristic_v1", "prob": 0.08}, {"name": "heuristic_v2", "prob": 0.12}, {"name": "random", "prob": 0.05}]</t>
+        </is>
+      </c>
+      <c r="N11" s="2">
+        <v>0</v>
+      </c>
+      <c r="O11" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2">
+        <v>20.52</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0.66</v>
+      </c>
+      <c r="R11" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>The 'definitive' 30M-game run vs the complete panel: PIMC-belief teacher 25%, value-lookahead 35%, mirror 15%, heuristics+random 25%, all on v9 base (panel doses by the maintainer). Beats v9 +0.66 head-to-head and sets a new all-time heuristic_v1 record (+20.52, up from 18.78): both progression meters at their maximum.</t>
+        </is>
+      </c>
+      <c r="T11" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T10"/>
+  <autoFilter ref="A1:T11"/>
 </worksheet>
 </file>
 
@@ -6062,7 +6528,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6803,59 +7269,140 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v10.npz</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/definitivo_vs_h1_big.json</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/definitivo_vs_v9_big.json</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B29" s="0" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D29" s="0" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E29"/>
+  <autoFilter ref="A1:E32"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(ai): promuovi v13 come nuovo default
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -24,6 +24,7 @@
     <sheet name="Detail best_a2c_v9" sheetId="16" r:id="rId16"/>
     <sheet name="Detail best_a2c_v10" sheetId="17" r:id="rId17"/>
     <sheet name="Detail best_a2c_v11" sheetId="18" r:id="rId18"/>
+    <sheet name="Detail best_a2c_v13" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -116,12 +117,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$15</c:f>
+              <c:f>Dashboard!$A$6:$A$16</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$15</c:f>
+              <c:f>Dashboard!$B$6:$B$16</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -137,12 +138,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$15</c:f>
+              <c:f>Dashboard!$A$6:$A$16</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$E$6:$E$15</c:f>
+              <c:f>Dashboard!$E$6:$E$16</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -235,7 +236,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -483,112 +484,106 @@
         <v>7.745</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="0" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>21.5182</v>
+      </c>
+      <c r="C16" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.1366</v>
+      </c>
+      <c r="E16" s="2">
+        <v>7.882</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>best_a2c_v10 is the recommended v0.27.0 .npz policy: a 30M-game run vs the complete panel (PIMC-belief teacher, value-lookahead, mirror, heuristics). It beats v9 (+0.66) and sets the all-time heuristic_v1 record (+20.52): both meters at their maximum. The value-lookahead runtime agent remains the stronger advanced option.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D23" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -598,7 +593,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D24" s="0">
@@ -606,14 +601,14 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -631,14 +626,14 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -656,14 +651,14 @@
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -677,18 +672,18 @@
         </is>
       </c>
       <c r="D27" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -706,14 +701,14 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.19.0 release.</t>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
+          <t>best_a2c_v7</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -723,7 +718,7 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D29" s="0">
@@ -731,14 +726,14 @@
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.22.0 release.</t>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v9</t>
+          <t>best_a2c_v8</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -752,18 +747,18 @@
         </is>
       </c>
       <c r="D30" s="0">
-        <v>20000000</v>
+        <v>5000000</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.26.0 release.</t>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v10</t>
+          <t>best_a2c_v9</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -777,36 +772,86 @@
         </is>
       </c>
       <c r="D31" s="0">
-        <v>30000000</v>
+        <v>20000000</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.27.0 release.</t>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
+          <t>best_a2c_v10</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D32" s="0">
+        <v>30000000</v>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v11</t>
         </is>
       </c>
-      <c r="B32" s="0" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>promoted</t>
         </is>
       </c>
-      <c r="C32" s="0" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>v4</t>
         </is>
       </c>
-      <c r="D32" s="0">
+      <c r="D33" s="0">
         <v>5000000</v>
       </c>
-      <c r="E32" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>Promoted as recommended model for the v0.31.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D34" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.34.0 release.</t>
         </is>
       </c>
     </row>
@@ -3517,9 +3562,309 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 (overkill shaping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_a2c_shaped_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260709</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v11.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_pimc_belief", "prob": 0.4}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.2}, {"name": "heuristic_trump_saver", "prob": 0.12}, {"name": "heuristic_v1", "prob": 0.04}, {"name": "heuristic_v2", "prob": 0.06}, {"name": "random", "prob": 0.03}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v11.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>21.5182</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>0.1366</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.34.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Overkill-shaping beta=0.3, warm-started from best_a2c_v11 for 5M games with a BC anchor toward v11. This is a behavior-cleanup promotion, not a strength-jump claim: policy-only v13 vs v11 is neutral (-0.03, CI -0.38..+0.32), and the default PIMC 16x8 gate is also neutral-slightly-positive (+0.14, CI -0.20..+0.47). The value is that low-lead trump overkill drops sharply (about 28-31% on v11 gates to 6-8% on v13) without breaking trump_saver or heuristic_v1 performance. Summary: same strength, better behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Promote v13 beta=0.3 as the recommended default model for v0.34.0.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>The overkill shaping changed the target behavior without measurable strength loss: same force as v11 within confidence intervals, much less low-lead trump overkill.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Policy-only v13 vs v11 -0.03 (CI -0.38..+0.32); default PIMC 16x8 v13 vs v11 +0.14 (CI -0.20..+0.47). Low-lead overkill drops from 27.8% to 6.1% vs v11 and from 31.4% to 7.8% vs heuristic_v1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E25"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4209,14 +4554,59 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Promote v13 beta=0.3 as the recommended default model for v0.34.0.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>The overkill shaping changed the target behavior without measurable strength loss: same force as v11 within confidence intervals, much less low-lead trump overkill.</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Policy-only v13 vs v11 -0.03 (CI -0.38..+0.32); default PIMC 16x8 v13 vs v11 +0.14 (CI -0.20..+0.47). Low-lead overkill drops from 27.8% to 6.1% vs v11 and from 31.4% to 7.8% vs heuristic_v1.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Default remains bc_model_pimc_belief_16x8, but now backed by best_a2c_v13.npz; no runtime overkill guard is reintroduced.</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz + v13_overkill_gap_beta0300_5M_seed20260709 gates</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I15"/>
+  <autoFilter ref="A1:I16"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:T13"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -5256,14 +5646,100 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 (overkill shaping)</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H13" s="0">
+        <v>369</v>
+      </c>
+      <c r="I13" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="J13" s="0">
+        <v>20260709</v>
+      </c>
+      <c r="K13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v11.npz</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>[{"name": "bc_model", "prob": 0.15}, {"name": "bc_model_pimc_belief", "prob": 0.4}, {"name": "bc_model_value_lookahead_8x8", "prob": 0.2}, {"name": "heuristic_trump_saver", "prob": 0.12}, {"name": "heuristic_v1", "prob": 0.04}, {"name": "heuristic_v2", "prob": 0.06}, {"name": "random", "prob": 0.03}]</t>
+        </is>
+      </c>
+      <c r="M13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v11.npz</t>
+        </is>
+      </c>
+      <c r="N13" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="O13" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2">
+        <v>21.5182</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0.1366</v>
+      </c>
+      <c r="R13" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.34.0 release.</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Overkill-shaping beta=0.3, warm-started from best_a2c_v11 for 5M games with a BC anchor toward v11. This is a behavior-cleanup promotion, not a strength-jump claim: policy-only v13 vs v11 is neutral (-0.03, CI -0.38..+0.32), and the default PIMC 16x8 gate is also neutral-slightly-positive (+0.14, CI -0.20..+0.47). The value is that low-lead trump overkill drops sharply (about 28-31% on v11 gates to 6-8% on v13) without breaking trump_saver or heuristic_v1 performance. Summary: same strength, better behavior.</t>
+        </is>
+      </c>
+      <c r="T13" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T12"/>
+  <autoFilter ref="A1:T13"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M26"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6487,14 +6963,274 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 policy</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v11_policy</t>
+        </is>
+      </c>
+      <c r="G22" s="2">
+        <v>-0.0272</v>
+      </c>
+      <c r="H22" s="0">
+        <v>4806</v>
+      </c>
+      <c r="I22" s="0">
+        <v>4910</v>
+      </c>
+      <c r="J22" s="0">
+        <v>284</v>
+      </c>
+      <c r="K22" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_v11_medium.json</t>
+        </is>
+      </c>
+      <c r="M22" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 policy</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G23" s="2">
+        <v>21.5182</v>
+      </c>
+      <c r="H23" s="0">
+        <v>7688</v>
+      </c>
+      <c r="I23" s="0">
+        <v>2124</v>
+      </c>
+      <c r="J23" s="0">
+        <v>188</v>
+      </c>
+      <c r="K23" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="M23" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 PIMC 16x8</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v11_pimc16x8</t>
+        </is>
+      </c>
+      <c r="G24" s="2">
+        <v>0.1366</v>
+      </c>
+      <c r="H24" s="0">
+        <v>4862</v>
+      </c>
+      <c r="I24" s="0">
+        <v>4815</v>
+      </c>
+      <c r="J24" s="0">
+        <v>323</v>
+      </c>
+      <c r="K24" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/pimc16x8_medium/v13_vs_v11_pimc16x8_medium.json</t>
+        </is>
+      </c>
+      <c r="M24" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 PIMC 16x8</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_trump_saver</t>
+        </is>
+      </c>
+      <c r="G25" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="H25" s="0">
+        <v>7262</v>
+      </c>
+      <c r="I25" s="0">
+        <v>2507</v>
+      </c>
+      <c r="J25" s="0">
+        <v>231</v>
+      </c>
+      <c r="K25" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/pimc16x8_medium/v13_vs_trumpsaver_pimc16x8_medium.json</t>
+        </is>
+      </c>
+      <c r="M25" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13 PIMC 16x8</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G26" s="2">
+        <v>22.4006</v>
+      </c>
+      <c r="H26" s="0">
+        <v>7807</v>
+      </c>
+      <c r="I26" s="0">
+        <v>1989</v>
+      </c>
+      <c r="J26" s="0">
+        <v>204</v>
+      </c>
+      <c r="K26" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/pimc16x8_medium/v13_vs_heuristic_v1_pimc16x8_medium.json</t>
+        </is>
+      </c>
+      <c r="M26" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M21"/>
+  <autoFilter ref="A1:M26"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6806,8 +7542,122 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v11</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v11</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G6" s="2">
+        <v>20.8664</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.001867356653</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.3001106544</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.3141430074</v>
+      </c>
+      <c r="K6" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/quality_v11_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="M6" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v13</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="G7" s="2">
+        <v>20.9396</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.001406606199</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.2209639607</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.07765667575</v>
+      </c>
+      <c r="K7" s="0">
+        <v>10000</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/quality_v13_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M5"/>
+  <autoFilter ref="A1:M7"/>
 </worksheet>
 </file>
 
@@ -6922,7 +7772,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E38"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -7825,59 +8675,140 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate</t>
+          <t>model</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>metadata_json read from .npz</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
+          <t>progress_metric</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>source for Dashboard progression score</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>h2h_metric</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/pimc16x8_medium/v13_vs_v11_pimc16x8_medium.json</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>source for head-to-head score</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
           <t>rejected_candidate</t>
         </is>
       </c>
-      <c r="B35" s="0" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>seed302_200k_conservative</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
-      <c r="D35" s="0" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E35"/>
+  <autoFilter ref="A1:E38"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(ai): promuovi v14 come modello predefinito
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -25,6 +25,7 @@
     <sheet name="Detail best_a2c_v10" sheetId="17" r:id="rId17"/>
     <sheet name="Detail best_a2c_v11" sheetId="18" r:id="rId18"/>
     <sheet name="Detail best_a2c_v13" sheetId="19" r:id="rId19"/>
+    <sheet name="Detail best_a2c_v14" sheetId="20" r:id="rId20"/>
   </sheets>
 </workbook>
 </file>
@@ -117,12 +118,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$9</c:f>
+              <c:f>Dashboard!$A$6:$A$10</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$9</c:f>
+              <c:f>Dashboard!$B$6:$B$10</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -215,7 +216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -383,112 +384,113 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>21.75808</v>
+      </c>
+      <c r="C10" s="0">
+        <v>100000</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>big 100k; standard seeds 0..49,999; seat-fair; Numba; promoted runtime config</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v13 is the recommended .npz policy in current v0.35.1 (first promoted in v0.34.0) and backs the default bc_model_pimc_belief_16x8 stack without an overkill guard. Its medium 10k gates show no material strength change from v11: policy-only -0.03 and PIMC 16x8 +0.14 head-to-head, both confidence intervals crossing zero. The promotion is behavioral: low-lead trump overkill falls from about 28-31% to 6-8%. v13 is excluded from the chart because no homogeneous big 100k result is available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v14 is the recommended .npz policy in current v0.36.0 and backs the default bc_model_pimc_belief_16x8 stack without an overkill guard. Distillation reduces suit-name argmax flips from 18.19% on v13 to 6.04%. Medium 10k gates show a small strength gain: policy-only +0.66 (CI +0.24..+1.09) and PIMC 16x8 +0.43 (CI +0.03..+0.84) against v13. The homogeneous big 100k control vs heuristic_v1 is +21.76, so v14 is included as the last chart row. v13 remains outside that chart because it has no big 100k result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D15" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E15" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D17" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -498,7 +500,7 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D18" s="0">
@@ -506,14 +508,14 @@
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -531,14 +533,14 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -556,14 +558,14 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -577,18 +579,18 @@
         </is>
       </c>
       <c r="D21" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -606,14 +608,14 @@
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.19.0 release.</t>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
+          <t>best_a2c_v7</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -623,7 +625,7 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D23" s="0">
@@ -631,14 +633,14 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.22.0 release.</t>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v9</t>
+          <t>best_a2c_v8</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -652,18 +654,18 @@
         </is>
       </c>
       <c r="D24" s="0">
-        <v>20000000</v>
+        <v>5000000</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.26.0 release.</t>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v10</t>
+          <t>best_a2c_v9</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -677,18 +679,18 @@
         </is>
       </c>
       <c r="D25" s="0">
-        <v>30000000</v>
+        <v>20000000</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.27.0 release.</t>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v11</t>
+          <t>best_a2c_v10</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -702,18 +704,18 @@
         </is>
       </c>
       <c r="D26" s="0">
-        <v>5000000</v>
+        <v>30000000</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.31.0 release.</t>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v13</t>
+          <t>best_a2c_v11</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -731,7 +733,57 @@
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
+          <t>Promoted as recommended model for the v0.31.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D28" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
           <t>Promoted as recommended model for the v0.34.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D29" s="0">
+        <v>50000</v>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.36.0 release.</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4090,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4908,14 +4960,375 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Promote the 50k suit-symmetry distillation as the recommended model for v0.36.0.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>The distilled policy keeps one normal forward pass while transferring most of the exact 24-view teacher's suit invariance and its playing-strength benefit.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Suit flips 18.19% -&gt; 6.04%; policy-only +0.66 vs v13 (CI +0.24..+1.09); default PIMC belief 16x8 +0.43 vs v13 (CI +0.03..+0.84); big 100k Numba +21.76 vs heuristic_v1.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Default remains bc_model_pimc_belief_16x8, now backed by best_a2c_v14.npz; inference cost and the no-guard runtime configuration remain unchanged.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>docs/plans/suit-distillation-v0-2026-07-11.md + suit_distillation_v0_50k_seed20260712 gates</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:I20"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E27"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v14.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14 (distillazione simmetrica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_bc_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260712</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>21.75808</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Progress protocol</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; big 100k; standard seeds; Numba; vs heuristic_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>0.6626</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>H2H protocol</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; medium 10k; suite medium; domain; vs best_a2c_v13</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.36.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>A single MLP distilled from the exact average of v13 logits over all 24 suit renamings, using 50k games and 1.9M labelled decisions. It reduces suit-dependent argmax flips from 18.19% to 6.04% while preserving decisiveness. It beats v13 policy-only by +0.66 (CI +0.24..+1.09) and in the real PIMC belief 16x8 stack by +0.43 (CI +0.03..+0.84). The homogeneous big 100k control vs heuristic_v1 reaches +21.76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Promote the 50k suit-symmetry distillation as the recommended model for v0.36.0.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>The distilled policy keeps one normal forward pass while transferring most of the exact 24-view teacher's suit invariance and its playing-strength benefit.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Suit flips 18.19% -&gt; 6.04%; policy-only +0.66 vs v13 (CI +0.24..+1.09); default PIMC belief 16x8 +0.43 vs v13 (CI +0.03..+0.84); big 100k Numba +21.76 vs heuristic_v1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E27"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6158,14 +6571,102 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v14.npz</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14 (distillazione simmetrica)</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H14" s="0">
+        <v>369</v>
+      </c>
+      <c r="I14" s="0">
+        <v>50000</v>
+      </c>
+      <c r="J14" s="0">
+        <v>20260712</v>
+      </c>
+      <c r="K14" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
+        </is>
+      </c>
+      <c r="L14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="P14" s="2">
+        <v>21.75808</v>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; big 100k; standard seeds; Numba; vs heuristic_v1</t>
+        </is>
+      </c>
+      <c r="R14" s="2">
+        <v>0.6626</v>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; medium 10k; suite medium; domain; vs best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="T14" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.36.0 release.</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>A single MLP distilled from the exact average of v13 logits over all 24 suit renamings, using 50k games and 1.9M labelled decisions. It reduces suit-dependent argmax flips from 18.19% to 6.04% while preserving decisiveness. It beats v13 policy-only by +0.66 (CI +0.24..+1.09) and in the real PIMC belief 16x8 stack by +0.43 (CI +0.03..+0.84). The homogeneous big 100k control vs heuristic_v1 reaches +21.76.</t>
+        </is>
+      </c>
+      <c r="V14" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V13"/>
+  <autoFilter ref="A1:V14"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R43"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -9203,14 +9704,236 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14 policy</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F41" s="0">
+        <v>0</v>
+      </c>
+      <c r="G41" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I41" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="K41" s="2">
+        <v>21.75808</v>
+      </c>
+      <c r="L41" s="0">
+        <v>77417</v>
+      </c>
+      <c r="M41" s="0">
+        <v>20561</v>
+      </c>
+      <c r="N41" s="0">
+        <v>2022</v>
+      </c>
+      <c r="O41" s="0">
+        <v>100000</v>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/39</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_v14_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="R41" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14 policy</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I42" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13_policy</t>
+        </is>
+      </c>
+      <c r="K42" s="2">
+        <v>0.6626</v>
+      </c>
+      <c r="L42" s="0">
+        <v>4990</v>
+      </c>
+      <c r="M42" s="0">
+        <v>4748</v>
+      </c>
+      <c r="N42" s="0">
+        <v>262</v>
+      </c>
+      <c r="O42" s="0">
+        <v>10000</v>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/40</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_vs_v13_medium.json</t>
+        </is>
+      </c>
+      <c r="R42" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14 PIMC 16x8</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t>bc_model_pimc_belief_16x8</t>
+        </is>
+      </c>
+      <c r="I43" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J43" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v13_pimc16x8</t>
+        </is>
+      </c>
+      <c r="K43" s="2">
+        <v>0.4342</v>
+      </c>
+      <c r="L43" s="0">
+        <v>4936</v>
+      </c>
+      <c r="M43" s="0">
+        <v>4758</v>
+      </c>
+      <c r="N43" s="0">
+        <v>306</v>
+      </c>
+      <c r="O43" s="0">
+        <v>10000</v>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/41</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/pimc16x8_vs_v13_medium.json</t>
+        </is>
+      </c>
+      <c r="R43" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R40"/>
+  <autoFilter ref="A1:R43"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -9762,8 +10485,81 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v14</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="K8" s="2">
+        <v>22.5112</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.0007389908535</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.2177371717</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0.04172423321</v>
+      </c>
+      <c r="O8" s="0">
+        <v>10000</v>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/decision_quality/6</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/quality_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="R8" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R7"/>
+  <autoFilter ref="A1:R8"/>
 </worksheet>
 </file>
 
@@ -10032,7 +10828,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E52"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -10206,34 +11002,34 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>stable_narrative</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>v14</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>data/models/bc_v3.npz</t>
+          <t>docs/plans/suit-distillation-v0-2026-07-11.md</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>curated_experiment_log</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>v14 suit-distillation pipeline, policy/PIMC gates, and promotion decision.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
@@ -10243,51 +11039,51 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>Not plotted: supervised teacher, not a playing baseline.</t>
+          <t>data/models/bc_v3.npz</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c.npz</t>
+          <t>Not plotted: supervised teacher, not a playing baseline.</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
@@ -10295,9 +11091,9 @@
           <t>best_a2c</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/matrix_big.json</t>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c.npz</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
@@ -10307,7 +11103,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10324,7 +11120,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/head_to_head_best_a2c_v2_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/matrix_big.json</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -10341,17 +11137,17 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
-        </is>
-      </c>
-      <c r="C12" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v3.npz</t>
+          <t>best_a2c</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/head_to_head_best_a2c_v2_big_numba.json</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -10361,14 +11157,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -10376,9 +11172,9 @@
           <t>best_a2c_v3</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/baseline_best_a2c_v3_big_vs_heuristic_v1_numba.json</t>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v3.npz</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -10388,7 +11184,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10405,7 +11201,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/best_a2c_v3_vs_best_a2c_2026-06-28_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/baseline_best_a2c_v3_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
@@ -10422,17 +11218,17 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
-        </is>
-      </c>
-      <c r="C15" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v4.npz</t>
+          <t>best_a2c_v3</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/best_a2c_v3_vs_best_a2c_2026-06-28_big_numba.json</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -10442,14 +11238,14 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -10457,9 +11253,9 @@
           <t>best_a2c_v4</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v4.npz</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -10469,7 +11265,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10486,7 +11282,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/head_to_head_best_a2c_v3_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -10503,17 +11299,17 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
-        </is>
-      </c>
-      <c r="C18" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v5.npz</t>
+          <t>best_a2c_v4</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/head_to_head_best_a2c_v3_big_numba.json</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -10523,14 +11319,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -10538,9 +11334,9 @@
           <t>best_a2c_v5</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
@@ -10550,7 +11346,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10567,7 +11363,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -10584,17 +11380,17 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v6.npz</t>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
@@ -10604,14 +11400,14 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -10619,9 +11415,9 @@
           <t>best_a2c_v6</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
@@ -10631,7 +11427,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10648,7 +11444,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
@@ -10665,17 +11461,17 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
-        </is>
-      </c>
-      <c r="C24" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v7.npz</t>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -10685,14 +11481,14 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -10700,9 +11496,9 @@
           <t>best_a2c_v7</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>data/eval_best_a2c_v7_vs_heuristic_v1_big_holdout_seedrange1000000.json</t>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -10712,7 +11508,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10729,7 +11525,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>data/eval_a2c_vs_value_lookahead_5M_vs_v6_big_holdout_seedrange1000000.json</t>
+          <t>data/eval_best_a2c_v7_vs_heuristic_v1_big_holdout_seedrange1000000.json</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
@@ -10746,17 +11542,17 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
-        </is>
-      </c>
-      <c r="C27" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v8.npz</t>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>data/eval_a2c_vs_value_lookahead_5M_vs_v6_big_holdout_seedrange1000000.json</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
@@ -10766,14 +11562,14 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -10781,9 +11577,9 @@
           <t>best_a2c_v8</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/iter2_h256_vs_heuristic_v1_big.json</t>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -10793,7 +11589,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10808,9 +11604,9 @@
           <t>best_a2c_v8</t>
         </is>
       </c>
-      <c r="C29" s="0" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/iter2_h256_vs_v7_big.json</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_heuristic_v1_big.json</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
@@ -10827,17 +11623,17 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v9</t>
+          <t>best_a2c_v8</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v9.npz</t>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_v7_big.json</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -10847,14 +11643,14 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -10864,7 +11660,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/superA_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v9.npz</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -10874,7 +11670,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10891,7 +11687,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/superA_vs_v8_big.json</t>
+          <t>benchmarks/experiments/fase3/superA_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
@@ -10908,17 +11704,17 @@
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v10</t>
+          <t>best_a2c_v9</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v10.npz</t>
+          <t>benchmarks/experiments/fase3/superA_vs_v8_big.json</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -10928,14 +11724,14 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -10945,7 +11741,7 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/definitivo_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v10.npz</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
@@ -10955,7 +11751,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -10972,7 +11768,7 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/definitivo_vs_v9_big.json</t>
+          <t>benchmarks/experiments/fase3/definitivo_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
@@ -10989,17 +11785,17 @@
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v11</t>
+          <t>best_a2c_v10</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v11.npz</t>
+          <t>benchmarks/experiments/fase3/definitivo_vs_v9_big.json</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
@@ -11009,14 +11805,14 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
@@ -11026,7 +11822,7 @@
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/v11_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v11.npz</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
@@ -11036,7 +11832,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11053,7 +11849,7 @@
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/v11_vs_v10_big.json</t>
+          <t>benchmarks/experiments/fase3/v11_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
@@ -11070,17 +11866,17 @@
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v13</t>
+          <t>best_a2c_v11</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v13.npz</t>
+          <t>benchmarks/experiments/fase3/v11_vs_v10_big.json</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
@@ -11090,14 +11886,14 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
@@ -11105,9 +11901,9 @@
           <t>best_a2c_v13</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
@@ -11117,7 +11913,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11930,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_v11_medium.json</t>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
@@ -11151,108 +11947,108 @@
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
+          <t>best_a2c_v13</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_v11_medium.json</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>seed302_200k_conservative</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v14.npz</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>pimc_distillation_v7</t>
-        </is>
-      </c>
-      <c r="C44" s="0" t="inlineStr">
-        <is>
-          <t>data/models/pimc_distill_v7_*.npz</t>
+          <t>best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_v14_vs_heuristic_v1_big_numba.json</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Expert-iteration probe: hard warm-start -2.33 vs v7; anchored variant -1.52; soft targets -9.19.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>exit_iter1b_belief_input</t>
+          <t>best_a2c_v14</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>data/models/exit_iter1b_a2c_v4belief_vs_vl_v7_5M_seed20260716.npz</t>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_vs_v13_medium.json</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Medium 10k: -0.56 vs its iter1 control (CI -1.05..-0.06); +0.82 vs v7.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
@@ -11264,12 +12060,12 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>pimc_teacher_v8_5m</t>
-        </is>
-      </c>
-      <c r="C46" s="0" t="inlineStr">
-        <is>
-          <t>data/models/pimc_teacher_v8_5M_32x10_seed20260721.npz</t>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
@@ -11279,7 +12075,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Big 100k: +0.40 vs v8, +16.71 vs heuristic_v1, and -0.63 vs the promoted mixed-panel arm.</t>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
         </is>
       </c>
     </row>
@@ -11291,12 +12087,12 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>v11_guard_on</t>
-        </is>
-      </c>
-      <c r="C47" s="0" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/v11guard_vs_v10_big.json</t>
+          <t>seed302_200k_conservative</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
@@ -11306,7 +12102,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Big 100k vs v10: +0.32 with guard, compared with +0.85 without it (about -0.53).</t>
+          <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
@@ -11318,27 +12114,135 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
+          <t>pimc_distillation_v7</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>data/models/pimc_distill_v7_*.npz</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Expert-iteration probe: hard warm-start -2.33 vs v7; anchored variant -1.52; soft targets -9.19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>exit_iter1b_belief_input</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>data/models/exit_iter1b_a2c_v4belief_vs_vl_v7_5M_seed20260716.npz</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Medium 10k: -0.56 vs its iter1 control (CI -1.05..-0.06); +0.82 vs v7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>pimc_teacher_v8_5m</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>data/models/pimc_teacher_v8_5M_32x10_seed20260721.npz</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Big 100k: +0.40 vs v8, +16.71 vs heuristic_v1, and -0.63 vs the promoted mixed-panel arm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>v11_guard_on</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/v11guard_vs_v10_big.json</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Big 100k vs v10: +0.32 with guard, compared with +0.85 without it (about -0.53).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v12</t>
         </is>
       </c>
-      <c r="C48" s="0" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>data/models/a2c_v12_saver12_pimc40_10M_seed20260708.npz</t>
         </is>
       </c>
-      <c r="D48" s="0" t="inlineStr">
+      <c r="D52" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>Big 100k: +0.11 vs v11 (CI -0.03..+0.25), +20.74 vs heuristic_v1; lead-load and trump-use profiles remained effectively unchanged.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E48"/>
+  <autoFilter ref="A1:E52"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(ai): promuove v15 come default efficiente
</commit_message>
<xml_diff>
--- a/docs/reports/model_progress.xlsx
+++ b/docs/reports/model_progress.xlsx
@@ -26,6 +26,7 @@
     <sheet name="Detail best_a2c_v11" sheetId="18" r:id="rId18"/>
     <sheet name="Detail best_a2c_v13" sheetId="19" r:id="rId19"/>
     <sheet name="Detail best_a2c_v14" sheetId="20" r:id="rId20"/>
+    <sheet name="Detail best_a2c_v15" sheetId="21" r:id="rId21"/>
   </sheets>
 </workbook>
 </file>
@@ -118,12 +119,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$6:$A$10</c:f>
+              <c:f>Dashboard!$A$6:$A$11</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$6:$B$10</c:f>
+              <c:f>Dashboard!$B$6:$B$11</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -216,7 +217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -410,112 +411,113 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>21.86688</v>
+      </c>
+      <c r="C11" s="0">
+        <v>100000</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>big 100k; standard seeds 0..49,999; seat-fair; Numba; promoted runtime config</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Current conclusion</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>best_a2c_v14 was promoted in v0.36.0 and remains the recommended .npz policy in current v0.37.0; it backs the default bc_model_pimc_belief_16x8 stack without an overkill guard. Distillation reduces suit-name argmax flips from 18.19% on v13 to 6.04%. Medium 10k gates show a small strength gain: policy-only +0.66 (CI +0.24..+1.09) and PIMC 16x8 +0.43 (CI +0.03..+0.84) against v13. The homogeneous big 100k control vs heuristic_v1 is +21.76, so v14 is included as the last chart row. v13 remains outside that chart because it has no big 100k result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t>Quick comparison</t>
-        </is>
-      </c>
-    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>best_a2c_v15 is the recommended .npz policy in current v0.38.0; it backs the default bc_model_pimc_belief_12x8 stack without an overkill guard. The 250k-game distillation transfers the exact 24-view average of the strongest 20M teacher into one compact policy. Policy-only v15 is +0.18 vs v14 on 100k paired games and +21.87 vs heuristic_v1 on the homogeneous big gate, so v15 is the last chart row. The runtime 12x8 gate is +0.11 vs v14 16x8 (CI -0.11..+0.32) on 20k games while mean and p95 search latency fall by about 25%. This is an efficiency/non-inferiority promotion, not a claim that 12x8 is statistically stronger. v13 remains outside the chart because it has no big 100k result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B16" s="0" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C16" s="0" t="inlineStr">
-        <is>
-          <t>Encoder</t>
-        </is>
-      </c>
-      <c r="D16" s="0" t="inlineStr">
-        <is>
-          <t>Training games</t>
-        </is>
-      </c>
-      <c r="E16" s="0" t="inlineStr">
-        <is>
-          <t>Decision</t>
+          <t>Quick comparison</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>teacher</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>Encoder</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Training games</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>promoted</t>
+          <t>teacher</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="D18" s="0">
-        <v>1000000</v>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
-          <t>Promoted as v2 best with overkill guard.</t>
+          <t>Use as BC teacher/anchor for v3 A2C runs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
+          <t>best_a2c</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -525,7 +527,7 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D19" s="0">
@@ -533,14 +535,14 @@
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended v3 baseline.</t>
+          <t>Promoted as v2 best with overkill guard.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
+          <t>best_a2c_v3</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -558,14 +560,14 @@
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended local/webapp/cloud model.</t>
+          <t>Promoted as recommended v3 baseline.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
+          <t>best_a2c_v4</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -583,14 +585,14 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.11.0 release.</t>
+          <t>Promoted as recommended local/webapp/cloud model.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
+          <t>best_a2c_v5</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -604,18 +606,18 @@
         </is>
       </c>
       <c r="D22" s="0">
-        <v>5000000</v>
+        <v>1000000</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.12.0 release.</t>
+          <t>Promoted as recommended model for the v0.11.0 release.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
+          <t>best_a2c_v6</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -633,14 +635,14 @@
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.19.0 release.</t>
+          <t>Promoted as recommended model for the v0.12.0 release.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
+          <t>best_a2c_v7</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -650,7 +652,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="D24" s="0">
@@ -658,14 +660,14 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.22.0 release.</t>
+          <t>Promoted as recommended model for the v0.19.0 release.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v9</t>
+          <t>best_a2c_v8</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -679,18 +681,18 @@
         </is>
       </c>
       <c r="D25" s="0">
-        <v>20000000</v>
+        <v>5000000</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.26.0 release.</t>
+          <t>Promoted as recommended model for the v0.22.0 release.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v10</t>
+          <t>best_a2c_v9</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -704,18 +706,18 @@
         </is>
       </c>
       <c r="D26" s="0">
-        <v>30000000</v>
+        <v>20000000</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.27.0 release.</t>
+          <t>Promoted as recommended model for the v0.26.0 release.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v11</t>
+          <t>best_a2c_v10</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -729,18 +731,18 @@
         </is>
       </c>
       <c r="D27" s="0">
-        <v>5000000</v>
+        <v>30000000</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.31.0 release.</t>
+          <t>Promoted as recommended model for the v0.27.0 release.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v13</t>
+          <t>best_a2c_v11</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -758,32 +760,82 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>Promoted as recommended model for the v0.34.0 release.</t>
+          <t>Promoted as recommended model for the v0.31.0 release.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D29" s="0">
+        <v>5000000</v>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>Promoted as recommended model for the v0.34.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v14</t>
         </is>
       </c>
-      <c r="B29" s="0" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>promoted</t>
         </is>
       </c>
-      <c r="C29" s="0" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>v4</t>
         </is>
       </c>
-      <c r="D29" s="0">
+      <c r="D30" s="0">
         <v>50000</v>
       </c>
-      <c r="E29" s="0" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>Promoted as recommended model for the v0.36.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D31" s="0">
+        <v>250000</v>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Promoted as the recommended model and 12x8 runtime for the v0.38.0 release.</t>
         </is>
       </c>
     </row>
@@ -4090,7 +4142,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -5005,8 +5057,53 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Promote the teacher-20M student with PIMC belief 12x8 as the v0.38.0 default.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>The larger suit-distillation transfers the 20M teacher into one compact policy, while 12x8 preserves the measured runtime strength of v14 16x8 at lower search cost.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Policy-only +0.18 vs v14 on 100k and +21.87 vs heuristic_v1 on the homogeneous big gate; runtime 12x8 vs v14 16x8 +0.11 (CI -0.11..+0.32) on 20k, with mean/p95 latency about 25% lower.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>The default becomes bc_model_pimc_belief_12x8(best_a2c_v15.npz). v14 16x8 and the older official models remain selectable; 64x10 remains the maximum-search option.</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>docs/diario/23-dodici-mondi-bastano.md + teacher20M 250k distillation and 12x8 gates</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
+  <autoFilter ref="A1:I21"/>
 </worksheet>
 </file>
 
@@ -5326,9 +5423,320 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E27"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Detail: best_a2c_v15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v15.npz</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Briscola AI v15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>mlp_bc_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Feature dim</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Training games</t>
+        </is>
+      </c>
+      <c r="B11" s="0">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B12" s="0">
+        <v>20260724</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Init</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Opponent mix</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BC anchor beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Guard anti-overkill</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Progress score</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>21.86688</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Progress protocol</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; big 100k; standard seeds; Numba; vs heuristic_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>H2H score</t>
+        </is>
+      </c>
+      <c r="B20" s="2">
+        <v>0.18046</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>H2H protocol</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; 100k; seed range 11,000,000; domain; vs best_a2c_v14</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Promoted as the recommended model and 12x8 runtime for the v0.38.0 release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>A 250k-game, 9.5M-decision student distilled from the exact 24-view suit average of the strongest 20M checkpoint. Policy-only it beats v14 by +0.18 on 100k paired games and reaches +21.87 in the homogeneous big control vs heuristic_v1. The release promotion is an efficiency decision: the real PIMC belief 12x8 stack is non-inferior to v14 16x8 (+0.11, CI -0.11..+0.32 on 20k games) while its mean and p95 search latency are about 25% lower. v14 16x8 remains selectable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>Decision milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Promote the teacher-20M student with PIMC belief 12x8 as the v0.38.0 default.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>The larger suit-distillation transfers the 20M teacher into one compact policy, while 12x8 preserves the measured runtime strength of v14 16x8 at lower search cost.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Policy-only +0.18 vs v14 on 100k and +21.87 vs heuristic_v1 on the homogeneous big gate; runtime 12x8 vs v14 16x8 +0.11 (CI -0.11..+0.32) on 20k, with mean/p95 latency about 25% lower.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E27"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -6659,14 +7067,97 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>official best</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>promoted</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v15.npz</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>Briscola AI v15</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="H15" s="0">
+        <v>369</v>
+      </c>
+      <c r="I15" s="0">
+        <v>250000</v>
+      </c>
+      <c r="J15" s="0">
+        <v>20260724</v>
+      </c>
+      <c r="L15" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>21.86688</v>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; big 100k; standard seeds; Numba; vs heuristic_v1</t>
+        </is>
+      </c>
+      <c r="R15" s="2">
+        <v>0.18046</v>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>policy, guard off; 100k; seed range 11,000,000; domain; vs best_a2c_v14</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Promoted as the recommended model and 12x8 runtime for the v0.38.0 release.</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>A 250k-game, 9.5M-decision student distilled from the exact 24-view suit average of the strongest 20M checkpoint. Policy-only it beats v14 by +0.18 on 100k paired games and reaches +21.87 in the homogeneous big control vs heuristic_v1. The release promotion is an efficiency decision: the real PIMC belief 12x8 stack is non-inferior to v14 16x8 (+0.11, CI -0.11..+0.32 on 20k games) while its mean and p95 search latency are about 25% lower. v14 16x8 remains selectable.</t>
+        </is>
+      </c>
+      <c r="V15" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V14"/>
+  <autoFilter ref="A1:V15"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R46"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -9926,14 +10417,224 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v15 policy</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>big</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>numba</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F44" s="0">
+        <v>0</v>
+      </c>
+      <c r="G44" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I44" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="K44" s="2">
+        <v>21.86688</v>
+      </c>
+      <c r="L44" s="0">
+        <v>77404</v>
+      </c>
+      <c r="M44" s="0">
+        <v>20522</v>
+      </c>
+      <c r="N44" s="0">
+        <v>2074</v>
+      </c>
+      <c r="O44" s="0">
+        <v>100000</v>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/42</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/eval_v15_vs_heuristic_v1_big_numba.json</t>
+        </is>
+      </c>
+      <c r="R44" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v15 policy</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F45" s="0">
+        <v>11000000</v>
+      </c>
+      <c r="G45" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I45" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J45" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14_policy</t>
+        </is>
+      </c>
+      <c r="K45" s="2">
+        <v>0.18046</v>
+      </c>
+      <c r="L45" s="0">
+        <v>48798</v>
+      </c>
+      <c r="M45" s="0">
+        <v>48317</v>
+      </c>
+      <c r="N45" s="0">
+        <v>2885</v>
+      </c>
+      <c r="O45" s="0">
+        <v>100000</v>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/43</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/confirm_student_vs_v14_100k.json</t>
+        </is>
+      </c>
+      <c r="R45" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v15 PIMC 12x8</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="G46" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H46" s="0" t="inlineStr">
+        <is>
+          <t>bc_model_pimc_belief_12x8</t>
+        </is>
+      </c>
+      <c r="I46" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v14_pimc16x8</t>
+        </is>
+      </c>
+      <c r="K46" s="2">
+        <v>0.1052</v>
+      </c>
+      <c r="L46" s="0">
+        <v>9689</v>
+      </c>
+      <c r="M46" s="0">
+        <v>9621</v>
+      </c>
+      <c r="N46" s="0">
+        <v>690</v>
+      </c>
+      <c r="O46" s="0">
+        <v>20000</v>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/promotion_evidence/44</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/efficiency_12x8/confirm_student12_vs_v14_16_20k.json</t>
+        </is>
+      </c>
+      <c r="R46" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R43"/>
+  <autoFilter ref="A1:R46"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R9"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -10558,8 +11259,81 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Best A2C v15</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>seat_fair</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>bc_model (direct policy)</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>heuristic_v1</t>
+        </is>
+      </c>
+      <c r="K9" s="2">
+        <v>22.493</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.0004092588803</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.2103586597</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0.01063684713</v>
+      </c>
+      <c r="O9" s="0">
+        <v>10000</v>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>docs/reports/evidence/model_progress.v1.json#/decision_quality/7</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/decision_quality_student_vs_heuristic_v1_medium.json</t>
+        </is>
+      </c>
+      <c r="R9" s="0" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R8"/>
+  <autoFilter ref="A1:R9"/>
 </worksheet>
 </file>
 
@@ -10828,7 +11602,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E56"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -11029,34 +11803,34 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>stable_narrative</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>bc_v3</t>
+          <t>v15</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>data/models/bc_v3.npz</t>
+          <t>docs/diario/23-dodici-mondi-bastano.md</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>curated_experiment_log</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>v15 teacher-20M distillation, 12x8 efficiency gate, release audit, and promotion decision.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
@@ -11066,51 +11840,51 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>Not plotted: supervised teacher, not a playing baseline.</t>
+          <t>data/models/bc_v3.npz</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>best_a2c</t>
+          <t>bc_v3</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c.npz</t>
+          <t>Not plotted: supervised teacher, not a playing baseline.</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
@@ -11118,9 +11892,9 @@
           <t>best_a2c</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/matrix_big.json</t>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c.npz</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -11130,7 +11904,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11921,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/head_to_head_best_a2c_v2_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/matrix_big.json</t>
         </is>
       </c>
       <c r="D12" s="0" t="inlineStr">
@@ -11164,17 +11938,17 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v3</t>
-        </is>
-      </c>
-      <c r="C13" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v3.npz</t>
+          <t>best_a2c</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v2_best_overkill_gap001_1m_seed50_numba/head_to_head_best_a2c_v2_big_numba.json</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -11184,14 +11958,14 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
@@ -11199,9 +11973,9 @@
           <t>best_a2c_v3</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/baseline_best_a2c_v3_big_vs_heuristic_v1_numba.json</t>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v3.npz</t>
         </is>
       </c>
       <c r="D14" s="0" t="inlineStr">
@@ -11211,7 +11985,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11228,7 +12002,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/best_a2c_v3_vs_best_a2c_2026-06-28_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/baseline_best_a2c_v3_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -11245,17 +12019,17 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v4</t>
-        </is>
-      </c>
-      <c r="C16" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v4.npz</t>
+          <t>best_a2c_v3</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/best_a2c_v3_vs_best_a2c_2026-06-28_big_numba.json</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
@@ -11265,14 +12039,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -11280,9 +12054,9 @@
           <t>best_a2c_v4</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v4.npz</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -11292,7 +12066,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11309,7 +12083,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/head_to_head_best_a2c_v3_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
@@ -11326,17 +12100,17 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v5</t>
-        </is>
-      </c>
-      <c r="C19" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v5.npz</t>
+          <t>best_a2c_v4</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_1m_numba/head_to_head_best_a2c_v3_big_numba.json</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
@@ -11346,14 +12120,14 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -11361,9 +12135,9 @@
           <t>best_a2c_v5</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v5.npz</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
@@ -11373,7 +12147,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11390,7 +12164,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/eval_big_vs_heuristic_v1_numba.json</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
@@ -11407,17 +12181,17 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v6</t>
-        </is>
-      </c>
-      <c r="C22" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v6.npz</t>
+          <t>best_a2c_v5</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v5_seed401_1m_numba/head_to_head_best_a2c_v4_big_numba.json</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
@@ -11427,14 +12201,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -11442,9 +12216,9 @@
           <t>best_a2c_v6</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v6.npz</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
@@ -11454,7 +12228,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11471,7 +12245,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_heuristic_v1_big_numba.json</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -11488,17 +12262,17 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v7</t>
-        </is>
-      </c>
-      <c r="C25" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v7.npz</t>
+          <t>best_a2c_v6</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v6_scaling_seed501_5m_numba/eval_5m_vs_best_a2c_v5_big_holdout_numba.json</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
@@ -11508,14 +12282,14 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -11523,9 +12297,9 @@
           <t>best_a2c_v7</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>data/eval_best_a2c_v7_vs_heuristic_v1_big_holdout_seedrange1000000.json</t>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v7.npz</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
@@ -11535,7 +12309,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11552,7 +12326,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>data/eval_a2c_vs_value_lookahead_5M_vs_v6_big_holdout_seedrange1000000.json</t>
+          <t>data/eval_best_a2c_v7_vs_heuristic_v1_big_holdout_seedrange1000000.json</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
@@ -11569,17 +12343,17 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v8</t>
-        </is>
-      </c>
-      <c r="C28" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v8.npz</t>
+          <t>best_a2c_v7</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>data/eval_a2c_vs_value_lookahead_5M_vs_v6_big_holdout_seedrange1000000.json</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
@@ -11589,14 +12363,14 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -11604,9 +12378,9 @@
           <t>best_a2c_v8</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/iter2_h256_vs_heuristic_v1_big.json</t>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v8.npz</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
@@ -11616,7 +12390,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11631,9 +12405,9 @@
           <t>best_a2c_v8</t>
         </is>
       </c>
-      <c r="C30" s="0" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/iter2_h256_vs_v7_big.json</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_heuristic_v1_big.json</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -11650,17 +12424,17 @@
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v9</t>
+          <t>best_a2c_v8</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v9.npz</t>
+          <t>benchmarks/experiments/fase3/iter2_h256_vs_v7_big.json</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -11670,14 +12444,14 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -11687,7 +12461,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/superA_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v9.npz</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
@@ -11697,7 +12471,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11714,7 +12488,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/superA_vs_v8_big.json</t>
+          <t>benchmarks/experiments/fase3/superA_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -11731,17 +12505,17 @@
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v10</t>
+          <t>best_a2c_v9</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v10.npz</t>
+          <t>benchmarks/experiments/fase3/superA_vs_v8_big.json</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
@@ -11751,14 +12525,14 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -11768,7 +12542,7 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/definitivo_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v10.npz</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
@@ -11778,7 +12552,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11795,7 +12569,7 @@
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/definitivo_vs_v9_big.json</t>
+          <t>benchmarks/experiments/fase3/definitivo_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D36" s="0" t="inlineStr">
@@ -11812,17 +12586,17 @@
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v11</t>
+          <t>best_a2c_v10</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v11.npz</t>
+          <t>benchmarks/experiments/fase3/definitivo_vs_v9_big.json</t>
         </is>
       </c>
       <c r="D37" s="0" t="inlineStr">
@@ -11832,14 +12606,14 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B38" s="0" t="inlineStr">
@@ -11849,7 +12623,7 @@
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/v11_vs_h1_big.json</t>
+          <t>data/models/best_a2c_v11.npz</t>
         </is>
       </c>
       <c r="D38" s="0" t="inlineStr">
@@ -11859,7 +12633,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11876,7 +12650,7 @@
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/fase3/v11_vs_v10_big.json</t>
+          <t>benchmarks/experiments/fase3/v11_vs_h1_big.json</t>
         </is>
       </c>
       <c r="D39" s="0" t="inlineStr">
@@ -11893,17 +12667,17 @@
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v13</t>
+          <t>best_a2c_v11</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
-          <t>data/models/best_a2c_v13.npz</t>
+          <t>benchmarks/experiments/fase3/v11_vs_v10_big.json</t>
         </is>
       </c>
       <c r="D40" s="0" t="inlineStr">
@@ -11913,14 +12687,14 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B41" s="0" t="inlineStr">
@@ -11928,9 +12702,9 @@
           <t>best_a2c_v13</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v13.npz</t>
         </is>
       </c>
       <c r="D41" s="0" t="inlineStr">
@@ -11940,7 +12714,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -11957,7 +12731,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_v11_medium.json</t>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_heuristic_v1_medium.json</t>
         </is>
       </c>
       <c r="D42" s="0" t="inlineStr">
@@ -11974,17 +12748,17 @@
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_model</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>best_a2c_v14</t>
-        </is>
-      </c>
-      <c r="C43" s="0" t="inlineStr">
-        <is>
-          <t>data/models/best_a2c_v14.npz</t>
+          <t>best_a2c_v13</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/v13_overkill_gap_beta0300_5M_seed20260709/eval_v13_vs_v11_medium.json</t>
         </is>
       </c>
       <c r="D43" s="0" t="inlineStr">
@@ -11994,14 +12768,14 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
-          <t>optional_raw_metric</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B44" s="0" t="inlineStr">
@@ -12009,9 +12783,9 @@
           <t>best_a2c_v14</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_v14_vs_heuristic_v1_big_numba.json</t>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v14.npz</t>
         </is>
       </c>
       <c r="D44" s="0" t="inlineStr">
@@ -12021,7 +12795,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Original metric audit input; not required to build the workbook.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12812,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_vs_v13_medium.json</t>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_v14_vs_heuristic_v1_big_numba.json</t>
         </is>
       </c>
       <c r="D45" s="0" t="inlineStr">
@@ -12055,108 +12829,108 @@
     <row r="46">
       <c r="A46" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>seed301_200k</t>
+          <t>best_a2c_v14</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
+          <t>benchmarks/experiments/suit_distillation_v0_50k_seed20260712/eval_vs_v13_medium.json</t>
         </is>
       </c>
       <c r="D46" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_model</t>
         </is>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>seed302_200k_conservative</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>data/models/best_a2c_v15.npz</t>
         </is>
       </c>
       <c r="D47" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
+          <t>Original metadata audit input; normalized fields are preserved in canonical_evidence.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>pimc_distillation_v7</t>
-        </is>
-      </c>
-      <c r="C48" s="0" t="inlineStr">
-        <is>
-          <t>data/models/pimc_distill_v7_*.npz</t>
+          <t>best_a2c_v15</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/eval_v15_vs_heuristic_v1_big_numba.json</t>
         </is>
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Expert-iteration probe: hard warm-start -2.33 vs v7; anchored variant -1.52; soft targets -9.19.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="0" t="inlineStr">
         <is>
-          <t>rejected_candidate_reference</t>
+          <t>optional_raw_metric</t>
         </is>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>exit_iter1b_belief_input</t>
+          <t>best_a2c_v15</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>data/models/exit_iter1b_a2c_v4belief_vs_vl_v7_5M_seed20260716.npz</t>
+          <t>benchmarks/experiments/suit_distillation_20m_teacher24_250k_seed20260724/confirm_student_vs_v14_100k.json</t>
         </is>
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>manual_summary</t>
+          <t>exact</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Medium 10k: -0.56 vs its iter1 control (CI -1.05..-0.06); +0.82 vs v7.</t>
+          <t>Original metric audit input; not required to build the workbook.</t>
         </is>
       </c>
     </row>
@@ -12168,12 +12942,12 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>pimc_teacher_v8_5m</t>
-        </is>
-      </c>
-      <c r="C50" s="0" t="inlineStr">
-        <is>
-          <t>data/models/pimc_teacher_v8_5M_32x10_seed20260721.npz</t>
+          <t>seed301_200k</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed301_200k_numba/model.npz</t>
         </is>
       </c>
       <c r="D50" s="0" t="inlineStr">
@@ -12183,7 +12957,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Big 100k: +0.40 vs v8, +16.71 vs heuristic_v1, and -0.63 vs the promoted mixed-panel arm.</t>
+          <t>big vs best_a2c_v3 +0.12/+0.13; decision-quality vs heuristic_v1 +16.91.</t>
         </is>
       </c>
     </row>
@@ -12195,12 +12969,12 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>v11_guard_on</t>
-        </is>
-      </c>
-      <c r="C51" s="0" t="inlineStr">
-        <is>
-          <t>benchmarks/experiments/fase3/v11guard_vs_v10_big.json</t>
+          <t>seed302_200k_conservative</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/a2c_v3_league_seed302_200k_conservative_numba/model.npz</t>
         </is>
       </c>
       <c r="D51" s="0" t="inlineStr">
@@ -12210,7 +12984,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Big 100k vs v10: +0.32 with guard, compared with +0.85 without it (about -0.53).</t>
+          <t>medium vs best_a2c_v3 -0.12/+0.05; vs heuristic_v1 +16.94/+16.95.</t>
         </is>
       </c>
     </row>
@@ -12222,27 +12996,135 @@
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
+          <t>pimc_distillation_v7</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>data/models/pimc_distill_v7_*.npz</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Expert-iteration probe: hard warm-start -2.33 vs v7; anchored variant -1.52; soft targets -9.19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>exit_iter1b_belief_input</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>data/models/exit_iter1b_a2c_v4belief_vs_vl_v7_5M_seed20260716.npz</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Medium 10k: -0.56 vs its iter1 control (CI -1.05..-0.06); +0.82 vs v7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>pimc_teacher_v8_5m</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>data/models/pimc_teacher_v8_5M_32x10_seed20260721.npz</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Big 100k: +0.40 vs v8, +16.71 vs heuristic_v1, and -0.63 vs the promoted mixed-panel arm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>v11_guard_on</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>benchmarks/experiments/fase3/v11guard_vs_v10_big.json</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>manual_summary</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Big 100k vs v10: +0.32 with guard, compared with +0.85 without it (about -0.53).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>rejected_candidate_reference</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
           <t>best_a2c_v12</t>
         </is>
       </c>
-      <c r="C52" s="0" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>data/models/a2c_v12_saver12_pimc40_10M_seed20260708.npz</t>
         </is>
       </c>
-      <c r="D52" s="0" t="inlineStr">
+      <c r="D56" s="0" t="inlineStr">
         <is>
           <t>manual_summary</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>Big 100k: +0.11 vs v11 (CI -0.03..+0.25), +20.74 vs heuristic_v1; lead-load and trump-use profiles remained effectively unchanged.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E52"/>
+  <autoFilter ref="A1:E56"/>
 </worksheet>
 </file>
 

</xml_diff>